<commit_message>
NPB自動更新(2軍): 2026-09-01 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-01/highlights_20260901.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-01/highlights_20260901.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7回裏にライトスタンドへ先制満塁ホームランを放ち、試合を決めた。</t>
+          <t>7回裏に先制満塁ホームランを放ち、試合の均衡を破る決勝打となった。</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3回と8回にそれぞれ本塁打を放ち、1試合2本塁打の活躍を見せた。</t>
+          <t>3回裏と8回裏に2本のホームランを放ち、チームの勝利に大きく貢献した。</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>延長10回裏にサヨナラタイムリーを放ち、チームを劇的な勝利に導いた。</t>
+          <t>10回裏にサヨナラタイムリーヒットを放ち、劇的な勝利をもたらした。</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9回表にレフトへ先制タイムリーを放ち、試合の均衡を破る決勝打となった。</t>
+          <t>9回表に代打で登場し、先制のタイムリーヒットを放ち試合を決めた。</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回表にセンターへ同点タイムリーツーベースを放ち、試合を振り出しに戻した。</t>
+          <t>7回表に同点タイムリーツーベースを放ち、試合の流れを大きく変えた。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>平山 功太</t>
+          <t>中村 奨成</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3回裏にレフトスタンドへ同点2ランを放ち、試合の流れを大きく変えた。</t>
+          <t>8回裏にダメ押しのソロホームランを放ち、チームの勝利を決定づけた。</t>
         </is>
       </c>
     </row>

</xml_diff>